<commit_message>
some bugs addressed in compute.py
</commit_message>
<xml_diff>
--- a/benchmark_prototype.xlsx
+++ b/benchmark_prototype.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\megha\Managing data for minor\Major\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13FFCB59-25E0-4ECA-9ADA-AAF40098AA95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9E86E109-2A57-4BC1-9010-A0A117463CC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="282" uniqueCount="229">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="280" uniqueCount="227">
   <si>
     <t>meta_data</t>
   </si>
@@ -1429,31 +1429,6 @@
     <t>Nikita and Order Statistics</t>
   </si>
   <si>
-    <t>Nikita likes tasks on order statistics, for example, he can easily find the k-th number in increasing order on a segment of an array. But now Nikita wonders how many segments of an array there are such that a given number x is the k-th number in increasing order on this segment. In other words, you should find the number of segments of a given array such that there are exactly k numbers of this segment which are less than x.
-Nikita wants to get answer for this question for each k from 0 to n, where n is the size of the array.
------Input-----
-The first line contains two integers n and x (1 &lt;= n &lt;= 2* 10^5, -10^9 &lt;= x &lt;= 10^9).
-The second line contains n integers a_1, a_2, ..., a_n (-10^9 &lt;= a_i &lt;= 10^9) — the given array.
------Output-----
-Print n+1 integers, where the i-th number is the answer for Nikita's question for k=i-1.
------Examples-----
-Input
-5 3
-1 2 3 4 5
-Output
-6 5 4 0 0 0
-Input
-2 6
--5 9
-Output
-1 2 0
-Input
-6 99
--1 -1 -1 -1 -1 -1
-Output
-0 6 5 4 3 2 1</t>
-  </si>
-  <si>
     <t>class Solution:
     def count_segments(self, n: int, x: int, arr: List[int]) -&gt; List[int]:</t>
   </si>
@@ -1462,44 +1437,6 @@
   </si>
   <si>
     <t>DZY Loves Planting</t>
-  </si>
-  <si>
-    <t>DZY loves planting, and he enjoys solving tree problems.
-DZY has a weighted tree (connected undirected graph without cycles) containing n nodes (they are numbered from 1 to n). He defines the function g(x, y) (1 ≤ x, y ≤ n) as the longest edge in the shortest path between nodes x and y. Specially g(z, z) = 0 for every z.
-For every integer sequence p_1, p_2, ..., p_n (1 ≤ p_i ≤ n), DZY defines f(p) as min_i = 1^n g(i, p_i).
-DZY wants to find such a sequence p that f(p) has maximum possible value. But there is one more restriction: the element j can appear in p at most x_j times.
-Please, find the maximum possible f(p) under the described restrictions.
------Input-----
-The first line contains an integer n (1 ≤ n ≤ 3000).
-Each of the next n - 1 lines contains three integers a_i, b_i, c_i (1 ≤ a_i, b_i ≤ n; 1 ≤ c_i ≤ 10000), denoting an edge between a_i and b_i with length c_i. It is guaranteed that these edges form a tree.
-Each of the next n lines describes an element of sequence x. The j-th line contains an integer x_j (1 ≤ x_j ≤ n).
------Output-----
-Print a single integer representing the answer.
------Examples-----
-Input
-4
-1 2 1
-2 3 2
-3 4 3
-1
-1
-1
-1
-Output
-2
-Input
-4
-1 2 1
-2 3 2
-3 4 3
-4
-4
-4
-4
-Output
-3
------Note-----
-In the first sample, one of the optimal p is [4, 3, 2, 1].</t>
   </si>
   <si>
     <t>class Solution:
@@ -1670,10 +1607,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -2182,7 +2122,7 @@
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="B11" t="s">
         <v>51</v>
@@ -2202,7 +2142,7 @@
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="B12" t="s">
         <v>55</v>
@@ -2222,7 +2162,7 @@
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="B13" t="s">
         <v>59</v>
@@ -2242,7 +2182,7 @@
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="B14" t="s">
         <v>63</v>
@@ -2262,7 +2202,7 @@
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="B15" t="s">
         <v>67</v>
@@ -2282,7 +2222,7 @@
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="B16" t="s">
         <v>71</v>
@@ -2302,7 +2242,7 @@
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="B17" t="s">
         <v>75</v>
@@ -2322,7 +2262,7 @@
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="B18" t="s">
         <v>79</v>
@@ -2342,7 +2282,7 @@
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="B19" t="s">
         <v>83</v>
@@ -2362,7 +2302,7 @@
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="B20" t="s">
         <v>75</v>
@@ -2382,7 +2322,7 @@
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="B21" t="s">
         <v>75</v>
@@ -2402,7 +2342,7 @@
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="B22" t="s">
         <v>93</v>
@@ -2422,7 +2362,7 @@
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="B23" t="s">
         <v>97</v>
@@ -2442,7 +2382,7 @@
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B24" t="s">
         <v>101</v>
@@ -2462,7 +2402,7 @@
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="B25" t="s">
         <v>105</v>
@@ -2482,7 +2422,7 @@
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="B26" t="s">
         <v>101</v>
@@ -2502,7 +2442,7 @@
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="B27" t="s">
         <v>109</v>
@@ -2522,7 +2462,7 @@
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B28" t="s">
         <v>113</v>
@@ -2542,7 +2482,7 @@
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="B29" t="s">
         <v>117</v>
@@ -2562,7 +2502,7 @@
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="B30" t="s">
         <v>121</v>
@@ -2582,7 +2522,7 @@
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="B31" t="s">
         <v>125</v>
@@ -2602,7 +2542,7 @@
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="B32" t="s">
         <v>125</v>
@@ -2622,7 +2562,7 @@
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="B33" t="s">
         <v>132</v>
@@ -2642,7 +2582,7 @@
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="B34" t="s">
         <v>136</v>
@@ -2662,7 +2602,7 @@
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="B35" t="s">
         <v>140</v>
@@ -2682,7 +2622,7 @@
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="B36" t="s">
         <v>144</v>
@@ -2702,7 +2642,7 @@
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="B37" t="s">
         <v>148</v>
@@ -2722,7 +2662,7 @@
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="B38" t="s">
         <v>152</v>
@@ -2742,7 +2682,7 @@
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="B39" t="s">
         <v>156</v>
@@ -2762,7 +2702,7 @@
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="B40" t="s">
         <v>160</v>
@@ -2782,7 +2722,7 @@
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="B41" t="s">
         <v>164</v>
@@ -2802,7 +2742,7 @@
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A42" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="B42" t="s">
         <v>168</v>
@@ -2822,7 +2762,7 @@
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B43" t="s">
         <v>172</v>
@@ -2842,7 +2782,7 @@
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="B44" t="s">
         <v>176</v>
@@ -2862,7 +2802,7 @@
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="B45" t="s">
         <v>180</v>
@@ -2882,7 +2822,7 @@
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="B46" t="s">
         <v>184</v>
@@ -2893,31 +2833,27 @@
       <c r="D46" t="s">
         <v>185</v>
       </c>
-      <c r="E46" t="s">
+      <c r="E46" s="2"/>
+      <c r="F46" t="s">
         <v>186</v>
-      </c>
-      <c r="F46" t="s">
-        <v>187</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="B47" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C47" t="s">
         <v>14</v>
       </c>
       <c r="D47" t="s">
+        <v>188</v>
+      </c>
+      <c r="E47" s="2"/>
+      <c r="F47" t="s">
         <v>189</v>
-      </c>
-      <c r="E47" t="s">
-        <v>190</v>
-      </c>
-      <c r="F47" t="s">
-        <v>191</v>
       </c>
     </row>
   </sheetData>

</xml_diff>